<commit_message>
refactor(audit): deterministic output + remove brittle Overview styling
- generated_at pinned to AUDIT_DATE (no wall-clock churn in JSON)
- Overview section headers styled by label match, not fixed cell coords
- drop unused datetime import / dead 'if False' branch
</commit_message>
<xml_diff>
--- a/audit/BMC-MAESTRO-AUDIT.xlsx
+++ b/audit/BMC-MAESTRO-AUDIT.xlsx
@@ -755,7 +755,7 @@
       <c r="B25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>DELTAS vs AUDITORÍA PREVIA</t>
         </is>
@@ -787,7 +787,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr"/>
       <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Repos hermanos: antes no enumerables -&gt; ahora 24 listados (solo 2 activos).</t>

</xml_diff>